<commit_message>
grafia BE THE DANCE  para minusculas
</commit_message>
<xml_diff>
--- a/translations Dance2Dance Ultima versao.xlsx
+++ b/translations Dance2Dance Ultima versao.xlsx
@@ -24452,11 +24452,11 @@
         <is>
           <t>Dançar é também encontrar o outro.
  Há músicas que nos fazem viajar, ritmos que despertam o corpo e movimentos que nos aproximam, mesmo quando não falamos a mesma língua.
- Be The Dance Day é um encontro aberto a todos, para dançar, divertir-se e partilhar a experiência do movimento ao som de diferentes músicas e culturas.
+ Be the Dance Day é um encontro aberto a todos, para dançar, divertir-se e partilhar a experiência do movimento ao som de diferentes músicas e culturas.
  Ao longo do encontro, somos convidados a experimentar diferentes ritmos, formas de dançar e maneiras de nos relacionarmos com a música e com quem está à nossa volta. Sem necessidade de saber dançar, sem passos certos ou errados, apenas a curiosidade de experimentar e a liberdade de nos deixarmos levar.
  Mais do que aprender uma dança, é uma oportunidade para viver a dança como encontro: com a música, com o corpo, com diferentes culturas e com outras pessoas.
  ​
- Be The Dance Day é uma celebração do movimento e da diversidade. Um espaço para soltar o corpo, descobrir novos ritmos, se divertir, criar conexões e simplesmente dançar.
+ Be the Dance Day é uma celebração do movimento e da diversidade. Um espaço para soltar o corpo, descobrir novos ritmos, se divertir, criar conexões e simplesmente dançar.
  Venha como você é. Vamos dançar juntos.</t>
         </is>
       </c>
@@ -24464,11 +24464,11 @@
         <is>
           <t>Dancing is also encountering the other.
 There is music that makes us travel, rhythms that awaken the body, and movements that bring us closer, even when we don't speak the same language.
-Be The Dance Day is an open gathering for everyone to dance, have fun, and share the experience of movement to the sounds of different music and cultures.
+Be the Dance Day is an open gathering for everyone to dance, have fun, and share the experience of movement to the sounds of different music and cultures.
 Throughout the gathering, we are invited to experience different rhythms, ways of dancing, and ways of relating to music and those around us. No dance experience is necessary, no right or wrong steps, just the curiosity to experiment and the freedom to let ourselves go.
 More than learning a dance, it is an opportunity to experience dance as an encounter: with music, with the body, with different cultures, and with other people.
 ​
-Be The Dance Day is a celebration of movement and diversity. A space to let the body loose, discover new rhythms, have fun, create connections, and simply dance.
+Be the Dance Day is a celebration of movement and diversity. A space to let the body loose, discover new rhythms, have fun, create connections, and simply dance.
 Come as you are. Let's dance together.</t>
         </is>
       </c>
@@ -24476,11 +24476,11 @@
         <is>
           <t>Å danse er også å møte den andre.
 Det finnes musikk som får oss til å reise, rytmer som vekker kroppen, og bevegelser som bringer oss nærmere hverandre, selv når vi ikke snakker samme språk.
-Be The Dance Day er en åpen samling for alle, for å danse, ha det gøy og dele opplevelsen av bevegelse til lyden av forskjellig musikk og kulturer.
+Be the Dance Day er en åpen samling for alle, for å danse, ha det gøy og dele opplevelsen av bevegelse til lyden av forskjellig musikk og kulturer.
 Gjennom samlingen inviteres vi til å oppleve ulike rytmer, måter å danse på, og måter å forholde oss til musikken og de rundt oss. Ingen danseerfaring er nødvendig, ingen riktige eller gale trinn, bare nysgjerrigheten til å eksperimentere og friheten til å la oss rive med.
 Mer enn å lære en dans, er det en mulighet til å oppleve dans som et møte: med musikk, med kroppen, med forskjellige kulturer, og med andre mennesker.
 ​
-Be The Dance Day er en feiring av bevegelse og mangfold. Et rom for å la kroppen delta, oppdage nye rytmer, ha det gøy, skape forbindelser, og rett og slett danse.
+Be the Dance Day er en feiring av bevegelse og mangfold. Et rom for å la kroppen delta, oppdage nye rytmer, ha det gøy, skape forbindelser, og rett og slett danse.
 Kom som du er. La oss danse sammen.</t>
         </is>
       </c>
@@ -24543,17 +24543,17 @@
       </c>
       <c r="D660" s="18" t="inlineStr">
         <is>
-          <t>BE THE DANCE DAY</t>
+          <t>Be the Dance Day</t>
         </is>
       </c>
       <c r="E660" s="18" t="inlineStr">
         <is>
-          <t>BE THE DANCE DAY</t>
+          <t>Be the Dance Day</t>
         </is>
       </c>
       <c r="F660" s="18" t="inlineStr">
         <is>
-          <t>BE THE DANCE DAY</t>
+          <t>Be the Dance Day</t>
         </is>
       </c>
       <c r="G660" s="5" t="inlineStr">
@@ -24584,10 +24584,10 @@
  O que é presença?
  Neste workshop, investigamos esse “algo mais”. Um convite para ir além da execução, do intelecto e da mente que observa e controla, e mergulhar numa experiência de presença, consciência e entrega.
  Através de práticas de educação somática, meditação, improvisação guiada e outras ferramentas de exploração do movimento, criamos espaço para escutar o corpo, ampliar a percepção e descobrir novas possibilidades de estar em cena.
- Mais do que acrescentar novas ferramentas à técnica, Be The Dance Pro propõe uma jornada para dentro de si. Uma investigação sobre o que acontece quando deixamos de apenas fazer a dança e permitimos que ela aconteça através de nós.
+ Mais do que acrescentar novas ferramentas à técnica, Be the Dance Pro propõe uma jornada para dentro de si. Uma investigação sobre o que acontece quando deixamos de apenas fazer a dança e permitimos que ela aconteça através de nós.
  O que é carisma?
  ​
- Be The Dance Pro é uma experiência de presença e totalidade. Um espaço para aprofundar a relação entre corpo, mente e movimento e descobrir aquilo que torna cada bailarino único. Uma busca por se perder na dança para encontrar aquele lugar onde bailarino e dança deixam de ser duas coisas diferentes.
+ Be the Dance Pro é uma experiência de presença e totalidade. Um espaço para aprofundar a relação entre corpo, mente e movimento e descobrir aquilo que torna cada bailarino único. Uma busca por se perder na dança para encontrar aquele lugar onde bailarino e dança deixam de ser duas coisas diferentes.
  O momento em que o bailarino é a própria dança.</t>
         </is>
       </c>
@@ -24598,10 +24598,10 @@
 What is presence?
 In this workshop, we investigate this “something more”. An invitation to go beyond execution, the intellect, and the mind that observes and controls, and dive into an experience of presence, awareness, and surrender.
 Through practices of somatic education, meditation, guided improvisation, and other tools for movement exploration, we create space to listen to the body, expand perception, and discover new possibilities of being on stage.
-More than adding new tools to technique, Be The Dance Pro proposes a journey inward. An investigation into what happens when we stop merely doing the dance and allow it to happen through us.
+More than adding new tools to technique, Be the Dance Pro proposes a journey inward. An investigation into what happens when we stop merely doing the dance and allow it to happen through us.
 What is charisma?
 ​
-Be The Dance Pro is an experience of presence and totality. A space to deepen the relationship between body, mind, and movement and discover what makes each dancer unique. A quest to lose oneself in the dance to find that place where dancer and dance cease to be two different things.
+Be the Dance Pro is an experience of presence and totality. A space to deepen the relationship between body, mind, and movement and discover what makes each dancer unique. A quest to lose oneself in the dance to find that place where dancer and dance cease to be two different things.
 The moment the dancer is the dance itself.</t>
         </is>
       </c>
@@ -24612,10 +24612,10 @@
 Hva er tilstedeværelse?
 I denne workshopen undersøker vi dette «noe mer». En invitasjon til å gå utover utførelse, intellektet og sinnet som observerer og kontrollerer, og dykke ned i en opplevelse av tilstedeværelse, bevissthet og overgivelse.
 Gjennom praksiser innen somatisk utdanning, meditasjon, veiledet improvisasjon og andre verktøy for bevegelsesutforskning, skaper vi rom for å lytte til kroppen, utvide persepsjonen og oppdage nye muligheter for å være på scenen.
-Mer enn å legge til nye verktøy til teknikken, foreslår Be The Dance Pro en reise innover. En undersøkelse av hva som skjer når vi slutter å bare gjøre dansen og lar den skje gjennom oss.
+Mer enn å legge til nye verktøy til teknikken, foreslår Be the Dance Pro en reise innover. En undersøkelse av hva som skjer når vi slutter å bare gjøre dansen og lar den skje gjennom oss.
 Hva er karisma?
 ​
-Be The Dance Pro er en opplevelse av tilstedeværelse og totalitet. Et rom for å utdype forholdet mellom kropp, sinn og bevegelse og oppdage hva som gjør hver danser unik. En søken etter å miste seg selv i dansen for å finne det stedet hvor danser og dans slutter å være to forskjellige ting.
+Be the Dance Pro er en opplevelse av tilstedeværelse og totalitet. Et rom for å utdype forholdet mellom kropp, sinn og bevegelse og oppdage hva som gjør hver danser unik. En søken etter å miste seg selv i dansen for å finne det stedet hvor danser og dans slutter å være to forskjellige ting.
 Øyeblikket hvor danseren er selve dansen.</t>
         </is>
       </c>
@@ -24678,17 +24678,17 @@
       </c>
       <c r="D663" s="19" t="inlineStr">
         <is>
-          <t>BE THE DANCE PRO</t>
+          <t>Be the Dance Pro</t>
         </is>
       </c>
       <c r="E663" s="19" t="inlineStr">
         <is>
-          <t>BE THE DANCE PRO</t>
+          <t>Be the Dance Pro</t>
         </is>
       </c>
       <c r="F663" s="19" t="inlineStr">
         <is>
-          <t>BE THE DANCE PRO</t>
+          <t>Be the Dance Pro</t>
         </is>
       </c>
       <c r="G663" s="9" t="inlineStr">

</xml_diff>

<commit_message>
excluido Bydel do bairro. agora é só Nabolag
</commit_message>
<xml_diff>
--- a/translations Dance2Dance Ultima versao.xlsx
+++ b/translations Dance2Dance Ultima versao.xlsx
@@ -6941,7 +6941,7 @@
       </c>
       <c r="D178" s="18" t="inlineStr">
         <is>
-          <t>Erro ao cancelar:</t>
+          <t xml:space="preserve">Erro ao cancelar: </t>
         </is>
       </c>
       <c r="E178" s="18" t="inlineStr">
@@ -9259,7 +9259,7 @@
       </c>
       <c r="F242" s="18" t="inlineStr">
         <is>
-          <t>Nabolag / Bydel *</t>
+          <t>Nabolag *</t>
         </is>
       </c>
       <c r="G242" s="5" t="inlineStr">
@@ -9499,7 +9499,11 @@
           <t>auth.phonePlaceholder</t>
         </is>
       </c>
-      <c r="D249" s="19" t="n"/>
+      <c r="D249" s="19" t="inlineStr">
+        <is>
+          <t>+55 ... / +47 ...</t>
+        </is>
+      </c>
       <c r="E249" s="19" t="inlineStr">
         <is>
           <t>+47 ...</t>
@@ -11578,12 +11582,12 @@
       </c>
       <c r="E306" s="18" t="inlineStr">
         <is>
-          <t>Automatic habits of movement: which were never chosen: become visible for the first time.</t>
+          <t>Automatic habits of movement - which were never chosen - become visible for the first time.</t>
         </is>
       </c>
       <c r="F306" s="18" t="inlineStr">
         <is>
-          <t>Automatiske bevegelsesvaner: som aldri ble valgt: blir synlige for første gang.</t>
+          <t>Automatiske bevegelsesvaner - som aldri ble valgt - blir synlige for første gang.</t>
         </is>
       </c>
       <c r="G306" s="5" t="inlineStr">
@@ -12947,8 +12951,10 @@
           <t>btd_corporate.pillars_section.pillars[0].number</t>
         </is>
       </c>
-      <c r="D344" s="18" t="n">
-        <v>1</v>
+      <c r="D344" s="18" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
       </c>
       <c r="E344" s="18" t="inlineStr">
         <is>
@@ -13233,8 +13239,10 @@
           <t>btd_corporate.pillars_section.pillars[1].number</t>
         </is>
       </c>
-      <c r="D352" s="18" t="n">
-        <v>2</v>
+      <c r="D352" s="18" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
       </c>
       <c r="E352" s="18" t="inlineStr">
         <is>
@@ -13519,8 +13527,10 @@
           <t>btd_corporate.pillars_section.pillars[2].number</t>
         </is>
       </c>
-      <c r="D360" s="18" t="n">
-        <v>3</v>
+      <c r="D360" s="18" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
       </c>
       <c r="E360" s="18" t="inlineStr">
         <is>
@@ -14709,7 +14719,11 @@
           <t>contactPage.phonePlaceholder</t>
         </is>
       </c>
-      <c r="D393" s="19" t="n"/>
+      <c r="D393" s="19" t="inlineStr">
+        <is>
+          <t>+55 ... / +47 ...</t>
+        </is>
+      </c>
       <c r="E393" s="19" t="inlineStr">
         <is>
           <t>+47 ...</t>
@@ -16733,8 +16747,10 @@
           <t>corporate.benefits.pillars[0].number</t>
         </is>
       </c>
-      <c r="D449" s="19" t="n">
-        <v>1</v>
+      <c r="D449" s="19" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
       </c>
       <c r="E449" s="19" t="inlineStr">
         <is>
@@ -17131,8 +17147,10 @@
           <t>corporate.benefits.pillars[1].number</t>
         </is>
       </c>
-      <c r="D460" s="18" t="n">
-        <v>2</v>
+      <c r="D460" s="18" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
       </c>
       <c r="E460" s="18" t="inlineStr">
         <is>
@@ -17533,8 +17551,10 @@
           <t>corporate.benefits.pillars[2].number</t>
         </is>
       </c>
-      <c r="D471" s="19" t="n">
-        <v>3</v>
+      <c r="D471" s="19" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
       </c>
       <c r="E471" s="19" t="inlineStr">
         <is>
@@ -22642,7 +22662,7 @@
       <c r="D611" s="19" t="inlineStr">
         <is>
           <t>[GOLD]Be The Dance. Não apenas dance.
- Seja a dança.</t>
+Seja a dança.</t>
         </is>
       </c>
       <c r="E611" s="19" t="inlineStr">
@@ -24217,9 +24237,9 @@
       <c r="D652" s="18" t="inlineStr">
         <is>
           <t>Encontrar o equilíbrio é aprender a escutar o corpo.
- O equilíbrio não é estático. Está em constante movimento, entre apoio e impulso, estabilidade e mudança, presença e ação.
- Neste workshop, exploramos essa relação dinâmica e as diferentes formas de encontrar estabilidade dentro do movimento. Um convite para descobrir como força, leveza e equilíbrio podem coexistir e criar novas possibilidades.
- O corpo possui uma inteligência própria. Quando aprendemos a escutá-lo, podemos confiar nas suas escolhas e permitir que ele encontre o seu próprio equilíbrio.</t>
+O equilíbrio não é estático. Está em constante movimento, entre apoio e impulso, estabilidade e mudança, presença e ação.
+Neste workshop, exploramos essa relação dinâmica e as diferentes formas de encontrar estabilidade dentro do movimento. Um convite para descobrir como força, leveza e equilíbrio podem coexistir e criar novas possibilidades.
+O corpo possui uma inteligência própria. Quando aprendemos a escutá-lo, podemos confiar nas suas escolhas e permitir que ele encontre o seu próprio equilíbrio.</t>
         </is>
       </c>
       <c r="E652" s="18" t="inlineStr">
@@ -24334,10 +24354,10 @@
       <c r="D655" s="19" t="inlineStr">
         <is>
           <t>Na quietude, o corpo começa a falar.
- Entre um pensamento e outro, entre uma respiração e a seguinte, existe o silêncio. É nesse intervalo que podemos escutar as sensações mais sutis do corpo.
- Neste workshop, exploramos a pausa e a escuta como parte essencial do movimento. Um convite para desacelerar e sentir o corpo, deixando surgir aquilo que se revela quando não há necessidade de estar sempre em movimento.
- A quietude não é ausência de movimento. É sobretudo possibilidade.
- Be Stillness é uma experiência de escuta. Um espaço para estar presente, encontrar o silêncio dentro do movimento e permitir que, a partir dele, a dança se revele.</t>
+Entre um pensamento e outro, entre uma respiração e a seguinte, existe o silêncio. É nesse intervalo que podemos escutar as sensações mais sutis do corpo.
+Neste workshop, exploramos a pausa e a escuta como parte essencial do movimento. Um convite para desacelerar e sentir o corpo, deixando surgir aquilo que se revela quando não há necessidade de estar sempre em movimento.
+A quietude não é ausência de movimento. É sobretudo possibilidade.
+Be Stillness é uma experiência de escuta. Um espaço para estar presente, encontrar o silêncio dentro do movimento e permitir que, a partir dele, a dança se revele.</t>
         </is>
       </c>
       <c r="E655" s="19" t="inlineStr">
@@ -24454,13 +24474,13 @@
       <c r="D658" s="18" t="inlineStr">
         <is>
           <t>Dançar é também encontrar o outro.
- Há músicas que nos fazem viajar, ritmos que despertam o corpo e movimentos que nos aproximam, mesmo quando não falamos a mesma língua.
- Be the Dance Day é um encontro aberto a todos, para dançar, divertir-se e partilhar a experiência do movimento ao som de diferentes músicas e culturas.
- Ao longo do encontro, somos convidados a experimentar diferentes ritmos, formas de dançar e maneiras de nos relacionarmos com a música e com quem está à nossa volta. Sem necessidade de saber dançar, sem passos certos ou errados, apenas a curiosidade de experimentar e a liberdade de nos deixarmos levar.
- Mais do que aprender uma dança, é uma oportunidade para viver a dança como encontro: com a música, com o corpo, com diferentes culturas e com outras pessoas.
- ​
- Be the Dance Day é uma celebração do movimento e da diversidade. Um espaço para soltar o corpo, descobrir novos ritmos, se divertir, criar conexões e simplesmente dançar.
- Venha como você é. Vamos dançar juntos.</t>
+Há músicas que nos fazem viajar, ritmos que despertam o corpo e movimentos que nos aproximam, mesmo quando não falamos a mesma língua.
+Be the Dance Day é um encontro aberto a todos, para dançar, divertir-se e partilhar a experiência do movimento ao som de diferentes músicas e culturas.
+Ao longo do encontro, somos convidados a experimentar diferentes ritmos, formas de dançar e maneiras de nos relacionarmos com a música e com quem está à nossa volta. Sem necessidade de saber dançar, sem passos certos ou errados, apenas a curiosidade de experimentar e a liberdade de nos deixarmos levar.
+Mais do que aprender uma dança, é uma oportunidade para viver a dança como encontro: com a música, com o corpo, com diferentes culturas e com outras pessoas.
+​
+Be the Dance Day é uma celebração do movimento e da diversidade. Um espaço para soltar o corpo, descobrir novos ritmos, se divertir, criar conexões e simplesmente dançar.
+Venha como você é. Vamos dançar juntos.</t>
         </is>
       </c>
       <c r="E658" s="18" t="inlineStr">
@@ -24583,15 +24603,15 @@
       <c r="D661" s="19" t="inlineStr">
         <is>
           <t>Você já é bailarino. Agora, seja a dança.
- A técnica é o instrumento através do qual o bailarino expressa a sua arte. Mas existe algo além dela: uma presença, uma qualidade de entrega, uma forma de estar no movimento que faz com que alguns bailarinos sejam capazes de capturar a nossa atenção e nos tocar de uma maneira única.
- O que é presença?
- Neste workshop, investigamos esse “algo mais”. Um convite para ir além da execução, do intelecto e da mente que observa e controla, e mergulhar numa experiência de presença, consciência e entrega.
- Através de práticas de educação somática, meditação, improvisação guiada e outras ferramentas de exploração do movimento, criamos espaço para escutar o corpo, ampliar a percepção e descobrir novas possibilidades de estar em cena.
- Mais do que acrescentar novas ferramentas à técnica, Be the Dance Pro propõe uma jornada para dentro de si. Uma investigação sobre o que acontece quando deixamos de apenas fazer a dança e permitimos que ela aconteça através de nós.
- O que é carisma?
- ​
- Be the Dance Pro é uma experiência de presença e totalidade. Um espaço para aprofundar a relação entre corpo, mente e movimento e descobrir aquilo que torna cada bailarino único. Uma busca por se perder na dança para encontrar aquele lugar onde bailarino e dança deixam de ser duas coisas diferentes.
- O momento em que o bailarino é a própria dança.</t>
+A técnica é o instrumento através do qual o bailarino expressa a sua arte. Mas existe algo além dela: uma presença, uma qualidade de entrega, uma forma de estar no movimento que faz com que alguns bailarinos sejam capazes de capturar a nossa atenção e nos tocar de uma maneira única.
+O que é presença?
+Neste workshop, investigamos esse “algo mais”. Um convite para ir além da execução, do intelecto e da mente que observa e controla, e mergulhar numa experiência de presença, consciência e entrega.
+Através de práticas de educação somática, meditação, improvisação guiada e outras ferramentas de exploração do movimento, criamos espaço para escutar o corpo, ampliar a percepção e descobrir novas possibilidades de estar em cena.
+Mais do que acrescentar novas ferramentas à técnica, Be the Dance Pro propõe uma jornada para dentro de si. Uma investigação sobre o que acontece quando deixamos de apenas fazer a dança e permitimos que ela aconteça através de nós.
+O que é carisma?
+​
+Be the Dance Pro é uma experiência de presença e totalidade. Um espaço para aprofundar a relação entre corpo, mente e movimento e descobrir aquilo que torna cada bailarino único. Uma busca por se perder na dança para encontrar aquele lugar onde bailarino e dança deixam de ser duas coisas diferentes.
+O momento em que o bailarino é a própria dança.</t>
         </is>
       </c>
       <c r="E661" s="19" t="inlineStr">
@@ -24790,10 +24810,10 @@
       <c r="D666" s="18" t="inlineStr">
         <is>
           <t>Dançar é ser inteiro. É não guardar nada.
- Sem se proteger, sem hesitar, sem guardar energia. Quando nos permitimos estar por inteiro no que fazemos, o corpo encontra liberdade para se expressar com espontaneidade e verdade.
- Neste workshop, exploramos a entrega total ao momento. Um convite para confiar no impulso, comprometer-se plenamente com cada gesto e deixar que o corpo se expresse sem reservas.
- Não se trata de fazer mais, mas de estar completamente presente no que fazemos. De colocar tudo no movimento e permitir que cada gesto seja vivido por inteiro.
- Be Total é uma experiência de entrega e expressão. Um espaço para estar totalmente presente, sem poupar energia e descobrir o que acontece quando nos permitimos dançar sem reservas.</t>
+Sem se proteger, sem hesitar, sem guardar energia. Quando nos permitimos estar por inteiro no que fazemos, o corpo encontra liberdade para se expressar com espontaneidade e verdade.
+Neste workshop, exploramos a entrega total ao momento. Um convite para confiar no impulso, comprometer-se plenamente com cada gesto e deixar que o corpo se expresse sem reservas.
+Não se trata de fazer mais, mas de estar completamente presente no que fazemos. De colocar tudo no movimento e permitir que cada gesto seja vivido por inteiro.
+Be Total é uma experiência de entrega e expressão. Um espaço para estar totalmente presente, sem poupar energia e descobrir o que acontece quando nos permitimos dançar sem reservas.</t>
         </is>
       </c>
       <c r="E666" s="18" t="inlineStr">
@@ -24982,10 +25002,10 @@
       <c r="D671" s="19" t="inlineStr">
         <is>
           <t>Entregar-se ao movimento é encontrar o fluxo.
- Quando deixamos de tentar conduzir cada gesto, o corpo encontra naturalmente novos caminhos. O movimento torna-se mais livre e orgânico, guiado pela escuta e pela sensação.
- Neste workshop, exploramos o fluir como possibilidade de expressão. Um convite para experimentar o movimento sem resistência, confiar no corpo e permitir que uma ação conduza naturalmente à seguinte.
- Como a água, que encontra o seu caminho sem precisar lutar contra ele, aprendemos a acompanhar o movimento em vez de controlá-lo.
- Be Water é uma experiência de entrega. Um espaço para deixar o corpo seguir o seu próprio fluxo e descobrir a dança que surge quando simplesmente nos deixamos levar.</t>
+Quando deixamos de tentar conduzir cada gesto, o corpo encontra naturalmente novos caminhos. O movimento torna-se mais livre e orgânico, guiado pela escuta e pela sensação.
+Neste workshop, exploramos o fluir como possibilidade de expressão. Um convite para experimentar o movimento sem resistência, confiar no corpo e permitir que uma ação conduza naturalmente à seguinte.
+Como a água, que encontra o seu caminho sem precisar lutar contra ele, aprendemos a acompanhar o movimento em vez de controlá-lo.
+Be Water é uma experiência de entrega. Um espaço para deixar o corpo seguir o seu próprio fluxo e descobrir a dança que surge quando simplesmente nos deixamos levar.</t>
         </is>
       </c>
       <c r="E671" s="19" t="inlineStr">
@@ -25826,7 +25846,7 @@
       <c r="D694" s="18" t="inlineStr">
         <is>
           <t>Talvez você tenha passado a vida inteira tentando fazer seu corpo obedecer.
- E se agora fosse o momento de escutá-lo? É essa investigação que proponho nas aulas de Biostretch. Um convite para desacelerar, para sentir, para respirar. Para soltar o que já não precisa ser sustentado. Para descobrir caminhos que estavam ali o tempo todo, esperando apenas que você prestasse atenção.</t>
+E se agora fosse o momento de escutá-lo? É essa investigação que proponho nas aulas de Biostretch. Um convite para desacelerar, para sentir, para respirar. Para soltar o que já não precisa ser sustentado. Para descobrir caminhos que estavam ali o tempo todo, esperando apenas que você prestasse atenção.</t>
         </is>
       </c>
       <c r="E694" s="18" t="inlineStr">
@@ -27309,11 +27329,11 @@
       <c r="D733" s="19" t="inlineStr">
         <is>
           <t>Estamos quase sempre ocupados com alguma coisa. Mas estar ocupado não significa, necessariamente, estar presente.
- Nosso corpo e nossa mente se acostumaram ao movimento, à ação e aos estímulos constantes. Por isso, simplesmente sentar, ficar em silêncio e estar presente pode ser um desafio.
- Vamos primeiro criar condições para que o corpo encontre conforto e quietude.
- No workshop Alongar, Respirar e Meditar, vamos explorar movimentos suaves para liberar as articulações e tensões desnecessárias. Vamos buscar pontos de apoio que nos permitam sentar com mais conforto e estabilidade, mantendo a coluna ereta sem rigidez.
- A respiração será nossa âncora enquanto o corpo e a mente desaceleram. Sem forçar. Sem tentar alcançar mais do que o corpo permite, apenas percebendo como o corpo está no momento.
- Sem precisar alcançar nada. Sem precisar fazer nada. Apenas criando espaço para a meditação acontecer.</t>
+Nosso corpo e nossa mente se acostumaram ao movimento, à ação e aos estímulos constantes. Por isso, simplesmente sentar, ficar em silêncio e estar presente pode ser um desafio.
+Vamos primeiro criar condições para que o corpo encontre conforto e quietude.
+No workshop Alongar, Respirar e Meditar, vamos explorar movimentos suaves para liberar as articulações e tensões desnecessárias. Vamos buscar pontos de apoio que nos permitam sentar com mais conforto e estabilidade, mantendo a coluna ereta sem rigidez.
+A respiração será nossa âncora enquanto o corpo e a mente desaceleram. Sem forçar. Sem tentar alcançar mais do que o corpo permite, apenas percebendo como o corpo está no momento.
+Sem precisar alcançar nada. Sem precisar fazer nada. Apenas criando espaço para a meditação acontecer.</t>
         </is>
       </c>
       <c r="E733" s="19" t="inlineStr">
@@ -27432,11 +27452,11 @@
       <c r="D736" s="18" t="inlineStr">
         <is>
           <t>Estar relaxado é nosso estado natural. Por isso, relaxar não é algo que possamos fazer, mas sim algo que podemos deixar acontecer liberando tensões e esforços que já não são necessários.
- Quando o corpo se sente seguro e confortável, o relaxamento acontece naturalmente e podemos perceber melhor nossa respiração, nossos movimentos e os hábitos que influenciam a maneira como nos relacionamos com o próprio corpo.
- ​
- No workshop Aprendendo a Relaxar, através de movimentos suaves e sem esforço, conectados com a respiração, vamos criar condições para que o corpo desacelere e o sistema nervoso encontre um estado de maior calma e restauração.
- O relaxamento se torna, então, muito mais do que uma pausa. Ele pode ser um caminho para ampliar a consciência, perceber o que acontece dentro de nós e descobrir novas possibilidades de estar no mundo.
- Mais calma por dentro. Mais presença, confiança e liberdade para encontrar o mundo lá fora.</t>
+Quando o corpo se sente seguro e confortável, o relaxamento acontece naturalmente e podemos perceber melhor nossa respiração, nossos movimentos e os hábitos que influenciam a maneira como nos relacionamos com o próprio corpo.
+​
+No workshop Aprendendo a Relaxar, através de movimentos suaves e sem esforço, conectados com a respiração, vamos criar condições para que o corpo desacelere e o sistema nervoso encontre um estado de maior calma e restauração.
+O relaxamento se torna, então, muito mais do que uma pausa. Ele pode ser um caminho para ampliar a consciência, perceber o que acontece dentro de nós e descobrir novas possibilidades de estar no mundo.
+Mais calma por dentro. Mais presença, confiança e liberdade para encontrar o mundo lá fora.</t>
         </is>
       </c>
       <c r="E736" s="18" t="inlineStr">
@@ -27555,10 +27575,10 @@
       <c r="D739" s="19" t="inlineStr">
         <is>
           <t>O estresse é uma resposta natural do nosso organismo diante de situações que exigem adaptação.
- A maneira como o nosso corpo responde ao estresse e retorna a um estado de equilíbrio, influencia nosso bem estar. Podemos permanecer por longos períodos acumulando tensão e esforço sem perceber. Com o tempo, isso pode afetar nossa energia, concentração, nosso sono, a capacidade de relaxar e nossa qualidade de vida.
- No workshop Movimentos Diários para Prevenir o Estresse, vamos explorar movimentos que ajudam a perceber e liberar tensões acumuladas e direcionar a atenção para regiões do corpo que tendemos a manter contraídas.
- Mais do que relaxar por alguns momentos, vamos aprender movimentos e estratégias simples que podem ser incorporados ao cotidiano, criando pequenas pausas para interromper o acúmulo de tensão e recuperar o equilíbrio.
- Aprender a perceber o estresse no corpo é o primeiro passo para aprender a responder a ele de uma maneira diferente.</t>
+A maneira como o nosso corpo responde ao estresse e retorna a um estado de equilíbrio, influencia nosso bem estar. Podemos permanecer por longos períodos acumulando tensão e esforço sem perceber. Com o tempo, isso pode afetar nossa energia, concentração, nosso sono, a capacidade de relaxar e nossa qualidade de vida.
+No workshop Movimentos Diários para Prevenir o Estresse, vamos explorar movimentos que ajudam a perceber e liberar tensões acumuladas e direcionar a atenção para regiões do corpo que tendemos a manter contraídas.
+Mais do que relaxar por alguns momentos, vamos aprender movimentos e estratégias simples que podem ser incorporados ao cotidiano, criando pequenas pausas para interromper o acúmulo de tensão e recuperar o equilíbrio.
+Aprender a perceber o estresse no corpo é o primeiro passo para aprender a responder a ele de uma maneira diferente.</t>
         </is>
       </c>
       <c r="E739" s="19" t="inlineStr">
@@ -27675,12 +27695,12 @@
       <c r="D742" s="18" t="inlineStr">
         <is>
           <t>Nosso foco está sendo roubado. Notificações, redes sociais, e-mails, multitarefas. Vivemos sob uma avalanche constante de informações que fragmenta nossa atenção e nos afasta do momento presente.
- Diante disso, é natural tentar recuperar a concentração com mais esforço: mais disciplina, mais controle, mais força de vontade. Mas a mente já está sobrecarregada. Exigir mais dela é como tentar esvaziar um copo cheio enchendo-o ainda mais.
- O caminho é inverso.
- Para recuperar a capacidade de foco, precisamos primeiro nos esvaziar. Liberar o acúmulo de tensão, de estímulos e de ruído que o corpo e a mente carregam sem perceber.
- No workshop Recuperando o Foco, vamos usar movimentos suaves e sem esforço para criar um espaço interno de silêncio e segurança. Ao direcionar a atenção para o corpo e para a respiração, permitimos que o sistema nervoso desacelere e que a mente encontre, naturalmente, um estado de maior clareza.
- Não se trata de treinar a concentração. Se trata de criar as condições para que ela se restaure por si mesma. Quando o corpo relaxa e a mente se esvazia, o foco ressurge como consequência de um estado de presença.
- Recuperar o foco é, antes de tudo, recuperar a quietude.</t>
+Diante disso, é natural tentar recuperar a concentração com mais esforço: mais disciplina, mais controle, mais força de vontade. Mas a mente já está sobrecarregada. Exigir mais dela é como tentar esvaziar um copo cheio enchendo-o ainda mais.
+O caminho é inverso.
+Para recuperar a capacidade de foco, precisamos primeiro nos esvaziar. Liberar o acúmulo de tensão, de estímulos e de ruído que o corpo e a mente carregam sem perceber.
+No workshop Recuperando o Foco, vamos usar movimentos suaves e sem esforço para criar um espaço interno de silêncio e segurança. Ao direcionar a atenção para o corpo e para a respiração, permitimos que o sistema nervoso desacelere e que a mente encontre, naturalmente, um estado de maior clareza.
+Não se trata de treinar a concentração. Se trata de criar as condições para que ela se restaure por si mesma. Quando o corpo relaxa e a mente se esvazia, o foco ressurge como consequência de um estado de presença.
+Recuperar o foco é, antes de tudo, recuperar a quietude.</t>
         </is>
       </c>
       <c r="E742" s="18" t="inlineStr">
@@ -27801,10 +27821,10 @@
       <c r="D745" s="19" t="inlineStr">
         <is>
           <t>Grande parte do que fazemos todos os dias acontece automaticamente. São hábitos e padrões de movimento que aprendemos ao longo da vida e que influenciam nossa postura, a maneira como nos movemos e até como nos sentimos.
- Os hábitos são importantes. Com eles, é possível realizar tarefas sem precisar reaprender a fazê-las a cada vez. Mas alguns padrões que um dia foram úteis podem, com o tempo, tornar-se limitantes, criando tensões, desconfortos e esforços desnecessários.
- No workshop Transformando Hábitos, vamos reconhecer esses padrões e experimentar novas possibilidades de movimento. Ao ampliar nossa percepção, surgem novos caminhos de movimento antes nunca usados.
- Um hábito não precisa simplesmente ser eliminado. Podemos transformá-lo, oferecendo ao corpo novas opções e permitindo que ele descubra maneiras mais fáceis, prazerosas e eficientes de se mover.
- Mais percepção. Mais possibilidades. Mais liberdade para escolher como se mover.</t>
+Os hábitos são importantes. Com eles, é possível realizar tarefas sem precisar reaprender a fazê-las a cada vez. Mas alguns padrões que um dia foram úteis podem, com o tempo, tornar-se limitantes, criando tensões, desconfortos e esforços desnecessários.
+No workshop Transformando Hábitos, vamos reconhecer esses padrões e experimentar novas possibilidades de movimento. Ao ampliar nossa percepção, surgem novos caminhos de movimento antes nunca usados.
+Um hábito não precisa simplesmente ser eliminado. Podemos transformá-lo, oferecendo ao corpo novas opções e permitindo que ele descubra maneiras mais fáceis, prazerosas e eficientes de se mover.
+Mais percepção. Mais possibilidades. Mais liberdade para escolher como se mover.</t>
         </is>
       </c>
       <c r="E745" s="19" t="inlineStr">
@@ -27921,12 +27941,12 @@
       <c r="D748" s="18" t="inlineStr">
         <is>
           <t>Sua postura conta uma história. Ela reflete a maneira como você organiza o corpo, os hábitos que desenvolveu ao longo da vida e a forma como se relaciona com o ambiente ao seu redor.
- Mais do que uma posição que devemos manter, a postura é uma organização dinâmica do corpo para se mover, se equilibrar e encontrar o mundo. Ela está presente em tudo o que fazemos e influencia nossa sensação de conforto, liberdade de movimento, apoio e bem-estar.
- Nosso esqueleto e nossa musculatura possuem uma incrível capacidade de nos sustentar contra a gravidade e, ao mesmo tempo, permitir movimento e adaptação. Porém, ao longo do tempo, podemos desenvolver hábitos que aumentam o esforço necessário para nos manter de pé e nos mover, criando tensão, desconforto e limitações desnecessárias.
- A postura não é, portanto, algo estático nem uma “posição correta” que precisamos controlar o tempo todo. As diferentes partes do corpo estão constantemente se relacionando e ajustando entre si. Existe uma conversa contínua entre músculos, ossos, respiração, equilíbrio e movimento.
- É essa inteligência inata do corpo que nos permite encontrar equilíbrio e suporte.
- No workshop Uma Melhor Postura, você terá a oportunidade de reconhecer padrões posturais habituais e explorar novas possibilidades de organização do corpo. Através da percepção e do movimento, podemos reduzir esforços desnecessários e descobrir maneiras mais eficazes, confortáveis e naturais de nos sustentar.
- Uma postura saudável não é rígida. Ela é estável e, ao mesmo tempo, flexível. É a sensação de estar apoiado, de encontrar a verticalidade sem esforço excessivo e de poder se mover com mais facilidade, liberdade e presença.</t>
+Mais do que uma posição que devemos manter, a postura é uma organização dinâmica do corpo para se mover, se equilibrar e encontrar o mundo. Ela está presente em tudo o que fazemos e influencia nossa sensação de conforto, liberdade de movimento, apoio e bem-estar.
+Nosso esqueleto e nossa musculatura possuem uma incrível capacidade de nos sustentar contra a gravidade e, ao mesmo tempo, permitir movimento e adaptação. Porém, ao longo do tempo, podemos desenvolver hábitos que aumentam o esforço necessário para nos manter de pé e nos mover, criando tensão, desconforto e limitações desnecessárias.
+A postura não é, portanto, algo estático nem uma “posição correta” que precisamos controlar o tempo todo. As diferentes partes do corpo estão constantemente se relacionando e ajustando entre si. Existe uma conversa contínua entre músculos, ossos, respiração, equilíbrio e movimento.
+É essa inteligência inata do corpo que nos permite encontrar equilíbrio e suporte.
+No workshop Uma Melhor Postura, você terá a oportunidade de reconhecer padrões posturais habituais e explorar novas possibilidades de organização do corpo. Através da percepção e do movimento, podemos reduzir esforços desnecessários e descobrir maneiras mais eficazes, confortáveis e naturais de nos sustentar.
+Uma postura saudável não é rígida. Ela é estável e, ao mesmo tempo, flexível. É a sensação de estar apoiado, de encontrar a verticalidade sem esforço excessivo e de poder se mover com mais facilidade, liberdade e presença.</t>
         </is>
       </c>
       <c r="E748" s="18" t="inlineStr">
@@ -28486,9 +28506,9 @@
           <t>programs.kroppsskole.subtitle</t>
         </is>
       </c>
-      <c r="D763" s="19" t="n"/>
-      <c r="E763" s="19" t="n"/>
-      <c r="F763" s="19" t="n"/>
+      <c r="D763" s="19" t="inlineStr"/>
+      <c r="E763" s="19" t="inlineStr"/>
+      <c r="F763" s="19" t="inlineStr"/>
       <c r="G763" s="11" t="inlineStr">
         <is>
           <t>Completo (3 idiomas) - Revisado nativo</t>
@@ -29349,7 +29369,7 @@
       <c r="D787" s="19" t="inlineStr">
         <is>
           <t>Porque o corpo não precisa apenas de estímulo.
- Precisa de tempo para aprender.</t>
+Precisa de tempo para aprender.</t>
         </is>
       </c>
       <c r="E787" s="19" t="inlineStr">
@@ -30655,17 +30675,17 @@
       </c>
       <c r="D823" s="19" t="inlineStr">
         <is>
-          <t>Gamle Oslo é um bairro de contrastes: diversidade, história e riqueza cultural convivem com desigualdades de acesso a serviços e atividades de qualidade. É exatamente esse contexto que nos chama a agir.</t>
+          <t>Tøyen e Grønland são bairros de contrastes - diversidade, história e riqueza cultural convivem com desigualdades de acesso a serviços e atividades de qualidade. É exatamente esse contexto que nos chama a agir.</t>
         </is>
       </c>
       <c r="E823" s="19" t="inlineStr">
         <is>
-          <t>Gamle Oslo is a neighbourhood of contrasts: diversity, history and cultural richness coexist with inequalities in access to quality services and activities. This is exactly the context that calls us to act.</t>
+          <t>Tøyen and Grønland are neighbourhoods of contrast - diversity, history and cultural richness coexist with inequalities in access to quality services and activities. This is exactly the context that calls us to act.</t>
         </is>
       </c>
       <c r="F823" s="19" t="inlineStr">
         <is>
-          <t>Gamle Oslo er et nabolag fylt av kontraster: mangfold, historie og kulturell rikdom eksisterer side om side med ulikhet i tilgang til kvalitetstjenester og aktiviteter. Det er nettopp denne virkeligheten som kaller oss til handling.</t>
+          <t>Tøyen og Grønland er nabolag fylt av kontraster - mangfold, historie og kulturell rikdom eksisterer side om side med ulikhet i tilgang til kvalitetstjenester og aktiviteter. Det er nettopp denne virkeligheten som kaller oss til handling.</t>
         </is>
       </c>
       <c r="G823" s="9" t="inlineStr">
@@ -30695,17 +30715,17 @@
       </c>
       <c r="D824" s="18" t="inlineStr">
         <is>
-          <t>O Dance2Dance nasce nesse território com uma missão clara: que a dança, a expressão corporal e o bem-estar não sejam privilégio de quem pode pagar. Cada workshop que desenvolvemos tem a mesma qualidade, o mesmo cuidado e a mesma intenção: independentemente de quem está na sala.</t>
+          <t>O Dance2Dance nasce nesse território com uma missão clara: que a dança, a expressão corporal e o bem-estar não sejam privilégio de quem pode pagar. Cada workshop que desenvolvemos tem a mesma qualidade, o mesmo cuidado e a mesma intenção - independentemente de quem está na sala.</t>
         </is>
       </c>
       <c r="E824" s="18" t="inlineStr">
         <is>
-          <t>Dance2Dance is born in this territory with a clear mission: that dance, movement and well-being should not be a privilege for those who can pay. Every workshop we develop carries the same quality, the same care and the same intention: regardless of who is in the room.</t>
+          <t>Dance2Dance is born in this territory with a clear mission: that dance, movement and well-being should not be a privilege for those who can pay. Every workshop we develop carries the same quality, the same care and the same intention - regardless of who is in the room.</t>
         </is>
       </c>
       <c r="F824" s="18" t="inlineStr">
         <is>
-          <t>Dance2Dance fødes i dette territoriet med et tydelig oppdrag: at dans, kroppsuttrykk og velvære ikke skal være et privilegium for dem som kan betale. Hver workshop vi utvikler har samme kvalitet, samme omsorg og samme intensjon: uavhengig av hvem som er i rommet.</t>
+          <t>Dance2Dance fødes i dette territoriet med et tydelig oppdrag: at dans, kroppsuttrykk og velvære ikke skal være et privilegium for dem som kan betale. Hver workshop vi utvikler har samme kvalitet, samme omsorg og samme intensjon - uavhengig av hvem som er i rommet.</t>
         </is>
       </c>
       <c r="G824" s="5" t="inlineStr">
@@ -30771,17 +30791,17 @@
       </c>
       <c r="D826" s="18" t="inlineStr">
         <is>
-          <t>Por que Gamle Oslo?</t>
+          <t>Por que Tøyen e Grønland?</t>
         </is>
       </c>
       <c r="E826" s="18" t="inlineStr">
         <is>
-          <t>Why Gamle Oslo?</t>
+          <t>Why Tøyen and Grønland?</t>
         </is>
       </c>
       <c r="F826" s="18" t="inlineStr">
         <is>
-          <t>Hvorfor Gamle Oslo?</t>
+          <t>Hvorfor Tøyen og Grønland?</t>
         </is>
       </c>
       <c r="G826" s="5" t="inlineStr">
@@ -30879,17 +30899,17 @@
       </c>
       <c r="D829" s="19" t="inlineStr">
         <is>
-          <t>Fundos, empresas e parceiros que chegam agora são parte da fundação: e da história: deste projeto. Entre em contato e descubra como fazer parte.</t>
+          <t>Fundos, empresas e parceiros que chegam agora são parte da fundação - e da história - deste projeto. Entre em contato e descubra como fazer parte.</t>
         </is>
       </c>
       <c r="E829" s="19" t="inlineStr">
         <is>
-          <t>Funds, companies and partners who arrive now are part of the foundation: and the story: of this project. Get in touch and discover how to be part of it.</t>
+          <t>Funds, companies and partners who arrive now are part of the foundation - and the story - of this project. Get in touch and discover how to be part of it.</t>
         </is>
       </c>
       <c r="F829" s="19" t="inlineStr">
         <is>
-          <t>Fond, bedrifter og partnere som kommer nå er en del av grunnlaget: og historien: til dette prosjektet. Ta kontakt og finn ut hvordan du kan være en del av det.</t>
+          <t>Fond, bedrifter og partnere som kommer nå er en del av grunnlaget - og historien - til dette prosjektet. Ta kontakt og finn ut hvordan du kan være en del av det.</t>
         </is>
       </c>
       <c r="G829" s="9" t="inlineStr">
@@ -31059,17 +31079,17 @@
       </c>
       <c r="D834" s="18" t="inlineStr">
         <is>
-          <t>Um modelo de acesso universal à cultura e ao movimento. Workshops de alto nível, gratuitos para moradores de Gamle Oslo: sustentados por múltiplas fontes de financiamento.</t>
+          <t>Um modelo de acesso universal à cultura e ao movimento. Workshops de alto nível, gratuitos para moradores de Tøyen e Grønland - sustentados por múltiplas fontes de financiamento.</t>
         </is>
       </c>
       <c r="E834" s="18" t="inlineStr">
         <is>
-          <t>A model for universal access to culture and movement. Premium workshops, free for residents of Gamle Oslo: sustained by multiple funding sources.</t>
+          <t>A model for universal access to culture and movement. Premium workshops, free for residents of Tøyen and Grønland - sustained by multiple funding sources.</t>
         </is>
       </c>
       <c r="F834" s="18" t="inlineStr">
         <is>
-          <t>En modell for universell tilgang til kultur og bevegelse. Premium workshops, gratis for beboere i Gamle Oslo: båret av flere finansieringskilder.</t>
+          <t>En modell for universell tilgang til kultur og bevegelse. Premium workshops, gratis for beboere i Tøyen og Grønland - båret av flere finansieringskilder.</t>
         </is>
       </c>
       <c r="G834" s="5" t="inlineStr">
@@ -31207,17 +31227,17 @@
       </c>
       <c r="D838" s="18" t="inlineStr">
         <is>
-          <t>O Dance2Dance foi desenhado para não depender de uma única fonte. Nossa sustentabilidade nasce da combinação estratégica de múltiplos pilares: cada um essencial, nenhum suficiente sozinho.</t>
+          <t>O Dance2Dance foi desenhado para não depender de uma única fonte. Nossa sustentabilidade nasce da combinação estratégica de múltiplos pilares - cada um essencial, nenhum suficiente sozinho.</t>
         </is>
       </c>
       <c r="E838" s="18" t="inlineStr">
         <is>
-          <t>Dance2Dance was designed not to rely on a single source. Our sustainability comes from the strategic combination of multiple pillars: each essential, none sufficient alone.</t>
+          <t>Dance2Dance was designed not to rely on a single source. Our sustainability comes from the strategic combination of multiple pillars - each essential, none sufficient alone.</t>
         </is>
       </c>
       <c r="F838" s="18" t="inlineStr">
         <is>
-          <t>Dance2Dance er designet for å ikke stole på en enkelt kilde. Vår bærekraft kommer fra den strategiske kombinasjonen av flere pilarer: hver enkelt essensiell, ingen tilstrekkelig alene.</t>
+          <t>Dance2Dance er designet for å ikke stole på en enkelt kilde. Vår bærekraft kommer fra den strategiske kombinasjonen av flere pilarer - hver enkelt essensiell, ingen tilstrekkelig alene.</t>
         </is>
       </c>
       <c r="G838" s="5" t="inlineStr">
@@ -31283,17 +31303,17 @@
       </c>
       <c r="D840" s="18" t="inlineStr">
         <is>
-          <t>Quem vem de fora de Gamle Oslo paga o valor real do workshop. Essa receita contribui diretamente para viabilizar o acesso gratuito aos moradores locais.</t>
+          <t>Quem vem de fora de Tøyen e Grønland paga o valor real do workshop. Essa receita contribui diretamente para viabilizar o acesso gratuito aos moradores locais.</t>
         </is>
       </c>
       <c r="E840" s="18" t="inlineStr">
         <is>
-          <t>Those who come from outside Gamle Oslo pay the real value of the workshop. This revenue directly contributes to enabling free access for local residents.</t>
+          <t>Those who come from outside Tøyen and Grønland pay the real value of the workshop. This revenue directly contributes to enabling free access for local residents.</t>
         </is>
       </c>
       <c r="F840" s="18" t="inlineStr">
         <is>
-          <t>De som kommer fra utenfor Gamle Oslo betaler den reelle verdien av workshopen. Denne inntekten bidrar direkte til å muliggjøre gratis tilgang for lokale beboere.</t>
+          <t>De som kommer fra utenfor Tøyen og Grønland betaler den reelle verdien av workshopen. Denne inntekten bidrar direkte til å muliggjøre gratis tilgang for lokale beboere.</t>
         </is>
       </c>
       <c r="G840" s="5" t="inlineStr">
@@ -31787,17 +31807,17 @@
       </c>
       <c r="D854" s="18" t="inlineStr">
         <is>
-          <t>Moradores de Gamle Oslo</t>
+          <t>Moradores de Tøyen e Grønland</t>
         </is>
       </c>
       <c r="E854" s="18" t="inlineStr">
         <is>
-          <t>Gamle Oslo residents</t>
+          <t>Tøyen and Grønland residents</t>
         </is>
       </c>
       <c r="F854" s="18" t="inlineStr">
         <is>
-          <t>Beboere i Gamle Oslo</t>
+          <t>Beboere i Tøyen og Grønland</t>
         </is>
       </c>
       <c r="G854" s="5" t="inlineStr">
@@ -31859,17 +31879,17 @@
       </c>
       <c r="D856" s="18" t="inlineStr">
         <is>
-          <t>“O acesso gratuito com transparência de preço cria dignidade. A pessoa não recebe caridade: recebe a oportunidade de participar de algo que tem valor real.”</t>
+          <t>“O acesso gratuito com transparência de preço cria dignidade. A pessoa não recebe caridade - recebe a oportunidade de participar de algo que tem valor real.”</t>
         </is>
       </c>
       <c r="E856" s="18" t="inlineStr">
         <is>
-          <t>“Free access with price transparency creates dignity. The person is not receiving charity: they are receiving the opportunity to be part of something with real value.”</t>
+          <t>“Free access with price transparency creates dignity. The person is not receiving charity - they are receiving the opportunity to be part of something with real value.”</t>
         </is>
       </c>
       <c r="F856" s="18" t="inlineStr">
         <is>
-          <t>“Gratis tilgang med pristransparens skaper verdighet. Personen mottar ikke veldedighet: de mottar muligheten til å være en del av noe med ekte verdi.”</t>
+          <t>“Gratis tilgang med pristransparens skaper verdighet. Personen mottar ikke veldedighet - de mottar muligheten til å være en del av noe med ekte verdi.”</t>
         </is>
       </c>
       <c r="G856" s="5" t="inlineStr">
@@ -31931,17 +31951,17 @@
       </c>
       <c r="D858" s="18" t="inlineStr">
         <is>
-          <t>Moradores de fora de Gamle Oslo participam mediante pagamento regular, com acesso à mesma experiência de qualidade premium.</t>
+          <t>Moradores de fora de Tøyen e Grønland participam mediante pagamento regular, com acesso à mesma experiência de qualidade premium.</t>
         </is>
       </c>
       <c r="E858" s="18" t="inlineStr">
         <is>
-          <t>Residents from outside Gamle Oslo participate at the regular rate, with access to the same premium quality experience.</t>
+          <t>Residents from outside Tøyen and Grønland participate at the regular rate, with access to the same premium quality experience.</t>
         </is>
       </c>
       <c r="F858" s="18" t="inlineStr">
         <is>
-          <t>Beboere utenfor Gamle Oslo deltar til vanlig pris, med tilgang til den samme premium-opplevelsen.</t>
+          <t>Beboere utenfor Tøyen og Grønland deltar til vanlig pris, med tilgang til den samme premium-opplevelsen.</t>
         </is>
       </c>
       <c r="G858" s="5" t="inlineStr">
@@ -32039,17 +32059,17 @@
       </c>
       <c r="D861" s="19" t="inlineStr">
         <is>
-          <t>Quem recebe gratuitamente recebe exatamente o mesmo que quem paga. Tornamos o preço real visível porque valor percebido importa: tanto para quem apia quanto para quem participa.</t>
+          <t>Quem recebe gratuitamente recebe exatamente o mesmo que quem paga. Tornamos o preço real visível porque valor percebido importa - tanto para quem apia quanto para quem participa.</t>
         </is>
       </c>
       <c r="E861" s="19" t="inlineStr">
         <is>
-          <t>Those who receive it for free receive exactly the same as those who pay. We make the real price visible because perceived value matters: for supporters and participants alike.</t>
+          <t>Those who receive it for free receive exactly the same as those who pay. We make the real price visible because perceived value matters - for supporters and participants alike.</t>
         </is>
       </c>
       <c r="F861" s="19" t="inlineStr">
         <is>
-          <t>De som mottar det gratis, mottar nøyaktig det samme som de som betaler. Vi gjør den reelle prisen synlig fordi opplevd verdi betyr noe: både for støttespillere og deltakere.</t>
+          <t>De som mottar det gratis, mottar nøyaktig det samme som de som betaler. Vi gjør den reelle prisen synlig fordi opplevd verdi betyr noe - både for støttespillere og deltakere.</t>
         </is>
       </c>
       <c r="G861" s="9" t="inlineStr">

</xml_diff>